<commit_message>
Update C++ standard to C++20; update dependencies.
</commit_message>
<xml_diff>
--- a/Data/StatsCLRTest.xlsx
+++ b/Data/StatsCLRTest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\Projects\C++\SoftwareInteroperability\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B43BD3-63C1-47B2-A573-CC3477158411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D009952E-5EC6-4B15-9267-56A6FDD84FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A02AB07-3C6C-4C2C-A3F0-E5C527E008B8}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{9A02AB07-3C6C-4C2C-A3F0-E5C527E008B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Basic Functionality" sheetId="1" r:id="rId1"/>
@@ -1010,6 +1010,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1017,7 +1018,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1666,6 +1666,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1673,7 +1674,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3236,7 +3236,7 @@
             <a:lstStyle/>
             <a:p>
               <a:r>
-                <a:rPr lang="en-US" sz="1100"/>
+                <a:rPr lang="en-GB" sz="1100"/>
                 <a:t>This chart isn't available in your version of Excel.
 Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
               </a:r>
@@ -3314,7 +3314,7 @@
             <a:lstStyle/>
             <a:p>
               <a:r>
-                <a:rPr lang="en-US" sz="1100"/>
+                <a:rPr lang="en-GB" sz="1100"/>
                 <a:t>This chart isn't available in your version of Excel.
 Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
               </a:r>
@@ -3329,9 +3329,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3369,7 +3369,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3475,7 +3475,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3617,7 +3617,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3692,7 +3692,7 @@
         <v>4.5</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I20" si="0">IF(ROUND(H3,6)-ROUND(F3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(H3,6)-ROUND(F3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K3" s="1" t="str">
@@ -3706,7 +3706,7 @@
         <v>6.5</v>
       </c>
       <c r="O3" t="str">
-        <f t="shared" ref="O3:O20" si="1">IF(ROUND(N3,6)-ROUND(L3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(N3,6)-ROUND(L3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q3" s="1" t="str">
@@ -3720,7 +3720,7 @@
         <v>4.5</v>
       </c>
       <c r="U3" t="str">
-        <f t="shared" ref="U3:U11" si="2">IF(ROUND(T3,6)-ROUND(R3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(T3,6)-ROUND(R3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
         <v>10</v>
       </c>
       <c r="I4" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H4,6)-ROUND(F4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K4" s="1" t="str">
@@ -3754,7 +3754,7 @@
         <v>10</v>
       </c>
       <c r="O4" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N4,6)-ROUND(L4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q4" s="1" t="str">
@@ -3767,7 +3767,7 @@
         <v>6.5</v>
       </c>
       <c r="U4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T4,6)-ROUND(R4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3788,7 +3788,7 @@
         <v>1.7757575757575756</v>
       </c>
       <c r="I5" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H5,6)-ROUND(F5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K5" s="1" t="str">
@@ -3801,7 +3801,7 @@
         <v>1.8477273941141912</v>
       </c>
       <c r="O5" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N5,6)-ROUND(L5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q5" s="13" t="str">
@@ -3814,7 +3814,7 @@
         <v>1.1696969696969697</v>
       </c>
       <c r="U5" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T5,6)-ROUND(R5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
         <v>-1.2242424242424244</v>
       </c>
       <c r="I6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H6,6)-ROUND(F6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K6" s="1" t="str">
@@ -3848,7 +3848,7 @@
         <v>-1.1522726058858088</v>
       </c>
       <c r="O6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N6,6)-ROUND(L6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q6" s="1" t="str">
@@ -3861,7 +3861,7 @@
         <v>82.5</v>
       </c>
       <c r="U6" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T6,6)-ROUND(R6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
         <v>9</v>
       </c>
       <c r="I7" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H7,6)-ROUND(F7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K7" s="1" t="str">
@@ -3895,7 +3895,7 @@
         <v>12</v>
       </c>
       <c r="O7" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N7,6)-ROUND(L7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q7" s="13" t="str">
@@ -3908,7 +3908,7 @@
         <v>1.2363636363636363</v>
       </c>
       <c r="U7" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T7,6)-ROUND(R7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H8,6)-ROUND(F8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K8" s="1" t="str">
@@ -3942,7 +3942,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N8,6)-ROUND(L8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q8" s="1" t="str">
@@ -3955,7 +3955,7 @@
         <v>96.5</v>
       </c>
       <c r="U8" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T8,6)-ROUND(R8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
         <v>2.25</v>
       </c>
       <c r="I9" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H9,6)-ROUND(F9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K9" s="1" t="str">
@@ -3989,7 +3989,7 @@
         <v>3.5</v>
       </c>
       <c r="O9" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N9,6)-ROUND(L9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q9" s="1" t="str">
@@ -4002,7 +4002,7 @@
         <v>118.5</v>
       </c>
       <c r="U9" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T9,6)-ROUND(R9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
         <v>4.5</v>
       </c>
       <c r="I10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H10,6)-ROUND(F10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K10" s="1" t="str">
@@ -4036,7 +4036,7 @@
         <v>7.5</v>
       </c>
       <c r="O10" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N10,6)-ROUND(L10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q10" s="1" t="str">
@@ -4049,7 +4049,7 @@
         <v>0.97598055237488623</v>
       </c>
       <c r="U10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T10,6)-ROUND(R10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4070,7 +4070,7 @@
         <v>4.5</v>
       </c>
       <c r="I11" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H11,6)-ROUND(F11,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K11" s="1" t="str">
@@ -4083,7 +4083,7 @@
         <v>7.5</v>
       </c>
       <c r="O11" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N11,6)-ROUND(L11,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="Q11" s="13" t="str">
@@ -4096,7 +4096,7 @@
         <v>0.952538038613988</v>
       </c>
       <c r="U11" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(T11,6)-ROUND(R11,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         <v>6.75</v>
       </c>
       <c r="I12" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H12,6)-ROUND(F12,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K12" s="1" t="str">
@@ -4130,7 +4130,7 @@
         <v>8.75</v>
       </c>
       <c r="O12" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N12,6)-ROUND(L12,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4145,7 +4145,7 @@
         <v>9</v>
       </c>
       <c r="I13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H13,6)-ROUND(F13,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K13" s="1" t="str">
@@ -4158,7 +4158,7 @@
         <v>11</v>
       </c>
       <c r="O13" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N13,6)-ROUND(L13,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H14,6)-ROUND(F14,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K14" s="1" t="str">
@@ -4186,7 +4186,7 @@
         <v>-0.17650417026049434</v>
       </c>
       <c r="O14" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N14,6)-ROUND(L14,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
         <v>2.8722813232690143</v>
       </c>
       <c r="I15" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H15,6)-ROUND(F15,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K15" s="1" t="str">
@@ -4214,7 +4214,7 @@
         <v>3.4423828956117011</v>
       </c>
       <c r="O15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N15,6)-ROUND(L15,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4229,7 +4229,7 @@
         <v>3.0276503540974917</v>
       </c>
       <c r="I16" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H16,6)-ROUND(F16,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K16" s="1" t="str">
@@ -4242,7 +4242,7 @@
         <v>3.6285901761795403</v>
       </c>
       <c r="O16" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N16,6)-ROUND(L16,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4257,7 +4257,7 @@
         <v>0.9574271077563381</v>
       </c>
       <c r="I17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H17,6)-ROUND(F17,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K17" s="1" t="str">
@@ -4270,7 +4270,7 @@
         <v>1.1474609652039003</v>
       </c>
       <c r="O17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N17,6)-ROUND(L17,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4285,7 +4285,7 @@
         <v>45</v>
       </c>
       <c r="I18" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H18,6)-ROUND(F18,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K18" s="1" t="str">
@@ -4298,7 +4298,7 @@
         <v>65</v>
       </c>
       <c r="O18" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N18,6)-ROUND(L18,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4313,7 +4313,7 @@
         <v>8.25</v>
       </c>
       <c r="I19" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H19,6)-ROUND(F19,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K19" s="1" t="str">
@@ -4326,7 +4326,7 @@
         <v>11.85</v>
       </c>
       <c r="O19" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N19,6)-ROUND(L19,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
         <v>9.1666666666666661</v>
       </c>
       <c r="I20" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H20,6)-ROUND(F20,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K20" s="1" t="str">
@@ -4354,7 +4354,7 @@
         <v>13.166666666666666</v>
       </c>
       <c r="O20" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(N20,6)-ROUND(L20,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
         <v>4.4408920985006264E-17</v>
       </c>
       <c r="I29" t="str">
-        <f t="shared" ref="I29:I41" si="3">IF(ROUND(H29,6)-ROUND(F29,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(H29,6)-ROUND(F29,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
         <v>9</v>
       </c>
       <c r="I30" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H30,6)-ROUND(F30,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
         <v>0</v>
       </c>
       <c r="I31" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H31,6)-ROUND(F31,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4510,7 +4510,7 @@
         <v>4.5</v>
       </c>
       <c r="I32" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H32,6)-ROUND(F32,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
         <v>9</v>
       </c>
       <c r="I33" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H33,6)-ROUND(F33,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
         <v>45</v>
       </c>
       <c r="I34" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H34,6)-ROUND(F34,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4570,7 +4570,7 @@
         <v>2.8722813232690143</v>
       </c>
       <c r="I35" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H35,6)-ROUND(F35,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4590,7 +4590,7 @@
         <v>3.0276503540974917</v>
       </c>
       <c r="I36" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H36,6)-ROUND(F36,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
         <v>0.9574271077563381</v>
       </c>
       <c r="I37" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H37,6)-ROUND(F37,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
         <v>8.25</v>
       </c>
       <c r="I38" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H38,6)-ROUND(F38,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
         <v>9.1666666666666661</v>
       </c>
       <c r="I39" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H39,6)-ROUND(F39,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4670,7 +4670,7 @@
         <v>2.25</v>
       </c>
       <c r="I40" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H40,6)-ROUND(F40,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
         <v>6.75</v>
       </c>
       <c r="I41" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ROUND(H41,6)-ROUND(F41,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4782,7 +4782,7 @@
         <v>#N/A</v>
       </c>
       <c r="G3" t="e">
-        <f t="shared" ref="G3:G17" si="0">IF(ROUND(F3,6)-ROUND(E3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(F3,6)-ROUND(E3,6)=0, "PASSED", "FAILED")</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
         <v>#N/A</v>
       </c>
       <c r="G4" t="e">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F4,6)-ROUND(E4,6)=0, "PASSED", "FAILED")</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -4815,11 +4815,11 @@
         <v>3</v>
       </c>
       <c r="F5" s="15">
-        <f t="shared" ref="F5:F17" si="1">AVERAGE(C3:C5)</f>
+        <f>AVERAGE(C3:C5)</f>
         <v>3</v>
       </c>
       <c r="G5" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F5,6)-ROUND(E5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4834,11 +4834,11 @@
         <v>5</v>
       </c>
       <c r="F6" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C4:C6)</f>
         <v>5</v>
       </c>
       <c r="G6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F6,6)-ROUND(E6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4853,11 +4853,11 @@
         <v>6.666666666666667</v>
       </c>
       <c r="F7" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C5:C7)</f>
         <v>6.666666666666667</v>
       </c>
       <c r="G7" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F7,6)-ROUND(E7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4872,11 +4872,11 @@
         <v>11</v>
       </c>
       <c r="F8" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C6:C8)</f>
         <v>11</v>
       </c>
       <c r="G8" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F8,6)-ROUND(E8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4891,11 +4891,11 @@
         <v>10</v>
       </c>
       <c r="F9" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C7:C9)</f>
         <v>10</v>
       </c>
       <c r="G9" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F9,6)-ROUND(E9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4910,11 +4910,11 @@
         <v>7.666666666666667</v>
       </c>
       <c r="F10" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C8:C10)</f>
         <v>7.666666666666667</v>
       </c>
       <c r="G10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F10,6)-ROUND(E10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4929,11 +4929,11 @@
         <v>3</v>
       </c>
       <c r="F11" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C9:C11)</f>
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F11,6)-ROUND(E11,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4948,11 +4948,11 @@
         <v>2.6666666666666665</v>
       </c>
       <c r="F12" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C10:C12)</f>
         <v>2.6666666666666665</v>
       </c>
       <c r="G12" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F12,6)-ROUND(E12,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4967,11 +4967,11 @@
         <v>4</v>
       </c>
       <c r="F13" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C11:C13)</f>
         <v>4</v>
       </c>
       <c r="G13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F13,6)-ROUND(E13,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -4986,11 +4986,11 @@
         <v>5</v>
       </c>
       <c r="F14" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C12:C14)</f>
         <v>5</v>
       </c>
       <c r="G14" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F14,6)-ROUND(E14,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5005,11 +5005,11 @@
         <v>5.666666666666667</v>
       </c>
       <c r="F15" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C13:C15)</f>
         <v>5.666666666666667</v>
       </c>
       <c r="G15" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F15,6)-ROUND(E15,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5024,11 +5024,11 @@
         <v>6</v>
       </c>
       <c r="F16" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C14:C16)</f>
         <v>6</v>
       </c>
       <c r="G16" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F16,6)-ROUND(E16,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5043,11 +5043,11 @@
         <v>6</v>
       </c>
       <c r="F17" s="15">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(C15:C17)</f>
         <v>6</v>
       </c>
       <c r="G17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(F17,6)-ROUND(E17,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5147,7 +5147,7 @@
         <v>2611.2838001159162</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I8" si="0">IF(ROUND(H3,6)-ROUND(F3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(H3,6)-ROUND(F3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K3" s="5" t="s">
@@ -5170,7 +5170,7 @@
         <v>-9.0783186977580819</v>
       </c>
       <c r="S3" t="str">
-        <f t="shared" ref="S3:S8" si="1">IF(ROUND(R3,6)-ROUND(P3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(R3,6)-ROUND(P3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U3" s="1">
@@ -5190,7 +5190,7 @@
         <v>-12.620591288724366</v>
       </c>
       <c r="AB3" t="str">
-        <f t="shared" ref="AB3:AB11" si="2">IF(ROUND(AA3,6)-ROUND(Y3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(AA3,6)-ROUND(Y3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5211,7 +5211,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H4,6)-ROUND(F4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K4" s="1"/>
@@ -5229,7 +5229,7 @@
         <v>7.9533834794647118E-6</v>
       </c>
       <c r="S4" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(R4,6)-ROUND(P4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U4" s="1">
@@ -5248,7 +5248,7 @@
         <v>5.2729354566083755E-30</v>
       </c>
       <c r="AB4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA4,6)-ROUND(Y4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
         <v>194</v>
       </c>
       <c r="I5" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H5,6)-ROUND(F5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K5" s="1"/>
@@ -5287,7 +5287,7 @@
         <v>9</v>
       </c>
       <c r="S5" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(R5,6)-ROUND(P5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U5" s="1">
@@ -5306,7 +5306,7 @@
         <v>30.481012658227847</v>
       </c>
       <c r="AB5" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA5,6)-ROUND(Y5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
         <v>9.2614599999999996</v>
       </c>
       <c r="I6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H6,6)-ROUND(F6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K6" s="1"/>
@@ -5345,7 +5345,7 @@
         <v>19.25</v>
       </c>
       <c r="S6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(R6,6)-ROUND(P6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U6" s="1">
@@ -5364,7 +5364,7 @@
         <v>326</v>
       </c>
       <c r="AB6" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA6,6)-ROUND(Y6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
         <v>2.278881E-2</v>
       </c>
       <c r="I7" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H7,6)-ROUND(F7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K7" s="1"/>
@@ -5397,7 +5397,7 @@
         <v>2.002914543026403</v>
       </c>
       <c r="S7" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(R7,6)-ROUND(P7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U7" s="1">
@@ -5416,7 +5416,7 @@
         <v>20.14457831325301</v>
       </c>
       <c r="AB7" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA7,6)-ROUND(Y7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
         <v>195</v>
       </c>
       <c r="I8" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(H8,6)-ROUND(F8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="K8" s="1"/>
@@ -5449,7 +5449,7 @@
         <v>10</v>
       </c>
       <c r="S8" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ROUND(R8,6)-ROUND(P8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
       <c r="U8" s="1">
@@ -5468,7 +5468,7 @@
         <v>6.414699343243238</v>
       </c>
       <c r="AB8" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA8,6)-ROUND(Y8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
         <v>249</v>
       </c>
       <c r="AB9" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA9,6)-ROUND(Y9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5520,7 +5520,7 @@
         <v>6.1077100486433737</v>
       </c>
       <c r="AB10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA10,6)-ROUND(Y10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -5546,7 +5546,7 @@
         <v>79</v>
       </c>
       <c r="AB11" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ROUND(AA11,6)-ROUND(Y11,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7296,7 +7296,7 @@
         <v>6.1280815146654328</v>
       </c>
       <c r="AB3" t="str">
-        <f t="shared" ref="AB3:AB10" si="0">IF(ROUND(AA3,6)-ROUND(Y3,6)=0, "PASSED", "FAILED")</f>
+        <f>IF(ROUND(AA3,6)-ROUND(Y3,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
         <v>0.4643666263162799</v>
       </c>
       <c r="AB4" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA4,6)-ROUND(Y4,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7412,7 +7412,7 @@
         <v>8.8945016827014396E-10</v>
       </c>
       <c r="AB5" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA5,6)-ROUND(Y5,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7470,7 +7470,7 @@
         <v>7.0181818181818167</v>
       </c>
       <c r="AB6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA6,6)-ROUND(Y6,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7522,7 +7522,7 @@
         <v>11</v>
       </c>
       <c r="AB7" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA7,6)-ROUND(Y7,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7550,7 +7550,7 @@
         <v>5.2625000000000002</v>
       </c>
       <c r="AB8" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA8,6)-ROUND(Y8,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7583,7 +7583,7 @@
         <v>0.70698050084244091</v>
       </c>
       <c r="AB9" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA9,6)-ROUND(Y9,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>
@@ -7609,7 +7609,7 @@
         <v>8</v>
       </c>
       <c r="AB10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ROUND(AA10,6)-ROUND(Y10,6)=0, "PASSED", "FAILED")</f>
         <v>PASSED</v>
       </c>
     </row>

</xml_diff>